<commit_message>
Add hyperlinked sources to timeline spreadsheet
Split Sources into 3 separate columns (Source 1, 2, 3) with each
source name as a clickable hyperlink to its URL.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Skyways_Timeline_Data.xlsx
+++ b/Skyways_Timeline_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Timeline Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Timeline Data'!$A$1:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Timeline Data'!$A$1:$K$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,12 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="7">
@@ -88,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -103,6 +109,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -470,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -479,9 +497,11 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="90" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -517,15 +537,25 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Source 1</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Source 2</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Source 3</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Highlight</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -562,17 +592,27 @@
           <t>Founding</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Fly Eye — Innovator Series; Crunchbase — Company Profile; The Drone Girl — Company Profile</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Fly Eye — Innovator Series</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Crunchbase — Company Profile</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>The Drone Girl — Company Profile</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -609,17 +649,23 @@
           <t>Milestone</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Crunchbase — Funding History; Fly Eye — CEO Interview</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Crunchbase — Funding History</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Fly Eye — CEO Interview</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -661,12 +707,14 @@
           <t>Skyways Internal — Not Published</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -703,17 +751,23 @@
           <t>Funding</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Crunchbase — Funding Rounds; The Drone Girl</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Crunchbase — Funding Rounds</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>The Drone Girl</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -750,17 +804,23 @@
           <t>Funding</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Crunchbase — Funding Rounds; The Drone Girl</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Crunchbase — Funding Rounds</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>The Drone Girl</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -797,17 +857,23 @@
           <t>Product</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Fly Eye — Technical Overview; Commercial UAV News</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Fly Eye — Technical Overview</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Commercial UAV News</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -849,12 +915,14 @@
           <t>Skyways Internal — Not Published</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -891,17 +959,23 @@
           <t>Contract — U.S. Navy</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>USNI News — Navy Drone Delivery; Commercial UAV News</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>USNI News — Navy Drone Delivery</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Commercial UAV News</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -938,17 +1012,23 @@
           <t>Product</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>sUAS News — V3 Announcement; Fly Eye — Aircraft Specs</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>sUAS News — V3 Announcement</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Fly Eye — Aircraft Specs</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -985,17 +1065,23 @@
           <t>Product</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>The Drone Girl; SBIR.gov — V2.5 referenced</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>The Drone Girl</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>SBIR.gov — V2.5 referenced</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="n"/>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1032,17 +1118,19 @@
           <t>Defense — U.S. Navy</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>USNI News — Feb 21, 2021 trials</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1079,17 +1167,19 @@
           <t>Contract — U.S. Air Force</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>SBIR.gov — Award FA8649-21-P-0539</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1126,17 +1216,23 @@
           <t>Contract — Commercial</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>SBIR.gov — Phase I references O&amp;G; The Drone Girl</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>SBIR.gov — Phase I references O&amp;G</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>The Drone Girl</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1173,17 +1269,19 @@
           <t>Defense</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>USNI News — Sea-Air-Space 2021</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1225,12 +1323,14 @@
           <t>Skyways Internal — Not Published</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1267,17 +1367,19 @@
           <t>Contract — U.S. Air Force</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>SBIR.gov — Skyways Portfolio</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1314,17 +1416,23 @@
           <t>Defense</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>NAVAIR — Official Release; DroneXL — Navy Drone Trials</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>NAVAIR — Official Release</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>DroneXL — Navy Drone Trials</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1361,17 +1469,27 @@
           <t>Defense — U.S. Navy / USMC</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>DVIDS — NAWCAD UAS Exercise; Inside Unmanned Systems; Navy.mil — FBP 23-1</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>DVIDS — NAWCAD UAS Exercise</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>Inside Unmanned Systems</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>Navy.mil — FBP 23-1</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1408,17 +1526,19 @@
           <t>Product</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>sUAS News — Skyways V3</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1455,17 +1575,23 @@
           <t>Defense</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>The Aviationist — RIMPAC; Battle Updates</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>The Aviationist — RIMPAC</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Battle Updates</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="n"/>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1502,17 +1628,19 @@
           <t>Contract — U.S. Air Force</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>SBIR.gov — $3,550,613 award</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1554,12 +1682,14 @@
           <t>Skyways Internal — Not Published</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1596,17 +1726,27 @@
           <t>Contract — U.S. Air Force</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Business Wire — Press Release; Skyways Newsroom; DRONELIFE</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Business Wire — Press Release</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Skyways Newsroom</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>DRONELIFE</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="K24" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1643,17 +1783,23 @@
           <t>Funding</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Business Wire; Skyways Newsroom</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Business Wire</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Skyways Newsroom</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1690,17 +1836,27 @@
           <t>Defense — DoD</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>Business Wire; Skyways Newsroom; DRONELIFE</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>Business Wire</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>Skyways Newsroom</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>DRONELIFE</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr">
+      <c r="K26" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1737,17 +1893,23 @@
           <t>Product</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>Skyways Newsroom; DroneXL</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Skyways Newsroom</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>DroneXL</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="n"/>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1784,17 +1946,23 @@
           <t>Product</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>DroneXL — Fleet Article; The Drone Girl</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>DroneXL — Fleet Article</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>The Drone Girl</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1831,17 +1999,27 @@
           <t>Contract — RWE (Germany)</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>GlobeNewswire; DroneXL; Energy Global</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>GlobeNewswire</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>DroneXL</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>Energy Global</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1878,17 +2056,23 @@
           <t>Contract — ANA Holdings (Japan)</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>The Drone Girl; Payload Asia</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>The Drone Girl</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Payload Asia</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="n"/>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1925,17 +2109,23 @@
           <t>Milestone</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>The Drone Girl — Inside Skyways; The Drone Girl — Roadmap</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>The Drone Girl — Inside Skyways</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>The Drone Girl — Roadmap</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1972,17 +2162,19 @@
           <t>Milestone</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>GlobeNewswire</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2019,17 +2211,23 @@
           <t>Milestone</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>Payload Asia; Japan Today</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Payload Asia</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>Japan Today</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2066,17 +2264,23 @@
           <t>Upcoming</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>DroneXL; ADrones</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>DroneXL</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>ADrones</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="n"/>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2113,24 +2317,90 @@
           <t>Upcoming</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>DroneXL; ADrones</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>DroneXL</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>ADrones</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="n"/>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I35"/>
+  <autoFilter ref="A1:K35"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId58"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>